<commit_message>
Data update incl. all Chinook from CTC
</commit_message>
<xml_diff>
--- a/data/TBRChinook_2024CatchApproximation.xlsx
+++ b/data/TBRChinook_2024CatchApproximation.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniepeacock/Library/CloudStorage/Dropbox-SalmonWatersheds/Stephanie Peacock/X Drive/1_PROJECTS/1_Active/State of Salmon/2_Data &amp; Analysis/state-of-salmon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F190FF2E-50AB-B04E-A000-3D0D6F211275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B3F93C-8788-9342-92CE-205007475868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3220" yWindow="1520" windowWidth="25640" windowHeight="14440" xr2:uid="{57D777E3-8A27-8C4F-B039-EC92A3CDBB96}"/>
+    <workbookView xWindow="38920" yWindow="3640" windowWidth="25640" windowHeight="14440" xr2:uid="{57D777E3-8A27-8C4F-B039-EC92A3CDBB96}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -532,11 +532,12 @@
         <v>2024</v>
       </c>
       <c r="C4" s="1">
-        <v>206</v>
+        <f>187+8</f>
+        <v>195</v>
       </c>
       <c r="D4" s="1">
-        <f>21*2</f>
-        <v>42</v>
+        <f>40</f>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -551,15 +552,15 @@
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C5" s="2">
         <f>SUM(C2:C4)</f>
-        <v>617</v>
+        <v>606</v>
       </c>
       <c r="D5" s="2">
         <f>SUM(D2:D4)</f>
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E5" s="2">
         <f>SUM(C5:D5)</f>
-        <v>730</v>
+        <v>717</v>
       </c>
       <c r="F5" t="s">
         <v>13</v>

</xml_diff>